<commit_message>
Leads: 2026-10-26 04:56 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-26.xlsx
+++ b/output/leads_2026-10-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -563,6 +563,62 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Elk River Plumbing &amp; Heating | Billings, MT</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>elkriverplumbingmt.com</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>https://elkriverplumbingmt.com/</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>elkriverplumbing@gmail.com</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>406-591-3810</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Billings MT</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>84</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>plumbing company Billings MT</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-26 05:02 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-26.xlsx
+++ b/output/leads_2026-10-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -584,7 +584,6 @@
           <t>https://elkriverplumbingmt.com/</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>elkriverplumbing@gmail.com</t>
@@ -614,6 +613,66 @@
         </is>
       </c>
       <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Maryland Sewer and Plumbing Service</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>mdsewer.com</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>https://www.mdsewer.com/plumbing/sewer-repair-in-annapolis</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>What Causes</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>info@mdsewer.com</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>410-255-9300</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Annapolis MD</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>100</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>sewer repair Annapolis MD</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-26 05:06 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-26.xlsx
+++ b/output/leads_2026-10-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -678,6 +678,66 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>In the Light Roofing</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>inthelightroofing.com</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>https://inthelightroofing.com/service-area/lehigh-valley/</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Services Across</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>info@inthelightroofing.com</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>(484) 553-0213</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Allentown PA</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>100</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>roof repair company Allentown PA</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-26 05:08 UTC (cycle 13)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-26.xlsx
+++ b/output/leads_2026-10-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -738,6 +738,66 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Odessa Roofing</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>odessaroofs.com</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>https://odessaroofs.com/</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Dependable Products</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>odessaroofing@aol.com</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>(859) 271-0524</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Lexington KY</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>90</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>roofing contractor Lexington KY</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-26 05:09 UTC (cycle 14)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-26.xlsx
+++ b/output/leads_2026-10-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -798,6 +798,66 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Lakewood Plumbing &amp; Heating</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>lakewoodplumbing.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>https://lakewoodplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Do You</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>scheduling@lakewoodheatingandcooling.com</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>303.233.7007</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Lakewood CO</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>100</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>plumber Lakewood CO</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-26 15:10 UTC (cycle 7)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-26.xlsx
+++ b/output/leads_2026-10-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -858,6 +858,122 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>No Time Flat Plumbing</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>notimeflatplumbing.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>https://notimeflatplumbing.com/</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Choice Than</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>admin@notimeflatplumbing.com</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>804.245.2179</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Richmond VA</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
+        <v>100</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>plumber Richmond VA</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>River City Plumbing — Richmond, VA Plumbers</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>rivercityplumb.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>https://rivercityplumb.com/</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>service@rivercityplumbing.com</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>(804) 555-0100</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Richmond VA</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>100</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>plumber Richmond VA</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-26 15:11 UTC (cycle 8)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-26.xlsx
+++ b/output/leads_2026-10-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -939,7 +939,6 @@
           <t>https://rivercityplumb.com/</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>service@rivercityplumbing.com</t>
@@ -969,6 +968,122 @@
         </is>
       </c>
       <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Action Sewer &amp; Septic Service, Inc</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>actionsewerseptic.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>https://www.actionsewerseptic.com/</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>info@actionsewerseptic.com</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>(319) 354-2784</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Iowa City IA</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
+        <v>100</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>sewer repair Iowa City IA</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>AC Guys Cooling &amp; Heating Services |</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ac-guys.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>https://ac-guys.com/air-conditioning-orlando/</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Kevin Harvey</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>acguys@ymail.com</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>(352) 242-0274</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Orlando FL</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>100</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>AC installation Orlando FL</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-26 15:13 UTC (cycle 9)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-26.xlsx
+++ b/output/leads_2026-10-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -994,7 +994,6 @@
           <t>https://www.actionsewerseptic.com/</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>info@actionsewerseptic.com</t>
@@ -1084,6 +1083,66 @@
         </is>
       </c>
       <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Emergency Plumber in Cary, NC | 24/7 Plumbing Services</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>proplumbingcary.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://proplumbingcary.com/</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>View Service</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>contact@proplumbingcary.com</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>(919) 944-7281</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Cary NC</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
+        <v>90</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>emergency plumber Cary NC</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-26 15:16 UTC (cycle 11)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-26.xlsx
+++ b/output/leads_2026-10-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1148,6 +1148,62 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>HVAC Companies Peoria, IL | Accurate Heating &amp; Cooling</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>accurate-heating.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://www.accurate-heating.com/</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>info@accurate-heating.com</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>(309) 249-5058</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Peoria IL</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
+        <v>100</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>air conditioning repair Peoria IL</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-26 15:17 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-26.xlsx
+++ b/output/leads_2026-10-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1169,7 +1169,6 @@
           <t>https://www.accurate-heating.com/</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>info@accurate-heating.com</t>
@@ -1199,6 +1198,66 @@
         </is>
       </c>
       <c r="L13" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>generalcontractordelaware.com</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>generalcontractordelaware.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>https://www.generalcontractordelaware.com/metal_roof.html</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Kent County</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>generalcontractordelaware@gmail.com</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>(302) 930-0811</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Dover DE</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>90</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Dover DE</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-26 15:22 UTC (cycle 15)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-26.xlsx
+++ b/output/leads_2026-10-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1263,6 +1263,66 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Drew Renovation</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>drewrenovation.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>https://drewrenovation.com/</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Enzo Tovar</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>drewrenovation@gmail.com</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>(828) 774-6941</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Asheville NC</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>100</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>roof repair company Asheville NC</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-26 15:23 UTC (cycle 16)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-26.xlsx
+++ b/output/leads_2026-10-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L15"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1323,6 +1323,62 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Capital 360</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>metalroofbaltimore.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>http://metalroofbaltimore.com/</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>moreinfo@metalroofbaltimore.com</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>(410) 287-3333</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Baltimore MD</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>84</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>metal roofing contractor Baltimore MD</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-26 20:57 UTC (cycle 1)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-26.xlsx
+++ b/output/leads_2026-10-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1344,7 +1344,6 @@
           <t>http://metalroofbaltimore.com/</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>moreinfo@metalroofbaltimore.com</t>
@@ -1374,6 +1373,62 @@
         </is>
       </c>
       <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Boulder Plumber</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>plumbingboulderco.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>https://www.plumbingboulderco.com/</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>info@plumbingboulderco.com</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>(720) 918-3388</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Boulder CO</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>100</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>plumbing company Boulder CO</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-26 21:01 UTC (cycle 4)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-26.xlsx
+++ b/output/leads_2026-10-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L17"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1399,7 +1399,6 @@
           <t>https://www.plumbingboulderco.com/</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>info@plumbingboulderco.com</t>
@@ -1429,6 +1428,62 @@
         </is>
       </c>
       <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>City Suburban Enviro Systems</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>citysuburban.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>https://www.citysuburban.com/</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>info@citysuburban.com</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>(315) 853-3899</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Utica NY</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>90</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>heating and cooling company Utica NY</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-26 21:03 UTC (cycle 5)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-26.xlsx
+++ b/output/leads_2026-10-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L18"/>
+  <dimension ref="A1:L19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1454,7 +1454,6 @@
           <t>https://www.citysuburban.com/</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>info@citysuburban.com</t>
@@ -1484,6 +1483,66 @@
         </is>
       </c>
       <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>The Arizona Roofer</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>thearizonaroofer.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>https://thearizonaroofer.com/best-roofing-contractor-chandler-az/</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Book Your</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>thearizonaroofer@gmail.com</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>(480) 435-5190</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Chandler AZ</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>100</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>roofing contractor Chandler AZ</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-26 21:04 UTC (cycle 6)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-26.xlsx
+++ b/output/leads_2026-10-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1548,6 +1548,66 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ApexGuard Roofing</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Roofing</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>apexguardroofing.repair</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>https://apexguardroofing.repair/</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Service Areas</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>info@apexguardroofing.repair</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>424-478-5284</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Torrance CA</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>100</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>roof repair company Torrance CA</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-26 21:10 UTC (cycle 10)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-26.xlsx
+++ b/output/leads_2026-10-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L20"/>
+  <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1608,6 +1608,62 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Maryland Sewer and Drain Pros</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Plumbing</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>marylandseweranddrainpros.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>https://www.marylandseweranddrainpros.com/service-areas/germantown</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>jerry@marylandseweranddrainpros.com</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>(227) 277-8138</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Germantown MD</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>100</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>sewer repair Germantown MD</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Leads: 2026-10-26 21:13 UTC (cycle 12)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-26.xlsx
+++ b/output/leads_2026-10-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L21"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1629,7 +1629,6 @@
           <t>https://www.marylandseweranddrainpros.com/service-areas/germantown</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>jerry@marylandseweranddrainpros.com</t>
@@ -1659,6 +1658,66 @@
         </is>
       </c>
       <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Polar Breeze</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>polarbreezeut.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>https://polarbreezeut.com/</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>System Was</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>info@polarbreezeut.com</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>(385) 292-7511</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Orem UT</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>90</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>air conditioning repair Orem UT</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
         <is>
           <t>2026-10-26</t>
         </is>

</xml_diff>

<commit_message>
Leads: 2026-10-26 21:16 UTC (cycle 14)
</commit_message>
<xml_diff>
--- a/output/leads_2026-10-26.xlsx
+++ b/output/leads_2026-10-26.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -1723,6 +1723,66 @@
         </is>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Breathe Clean Air Conditioning &amp; Heating Repair</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>HVAC</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>breathecleanairconditioning.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>https://breathecleanairconditioning.com/locations/bellingham-wa.html</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Why Bellingham</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>service@breathecleanairconditioning.com</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>(888) 691-5826</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Bellingham WA</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>90</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>air conditioning repair Bellingham WA</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>ddg</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-10-26</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>